<commit_message>
fixed loaddata and ship functionality from admin page
</commit_message>
<xml_diff>
--- a/projectMarkingSoFar.xlsx
+++ b/projectMarkingSoFar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soljt\Documents\COSC 304\cosc304-project-group1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55590046-DA4C-4E20-9DB9-71D347628A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F69C6E6-625F-465E-B360-88C6E1AC4606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{24B39AA9-47B0-4981-9C08-9EA32D2EDF33}"/>
   </bookViews>
@@ -428,6 +428,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -454,21 +469,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -808,13 +808,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="13"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -841,7 +841,9 @@
       <c r="C4" s="6">
         <v>2</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="7">
+        <v>2</v>
+      </c>
       <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -854,24 +856,26 @@
       <c r="C5" s="6">
         <v>6</v>
       </c>
-      <c r="D5" s="7"/>
+      <c r="D5" s="7">
+        <v>6</v>
+      </c>
       <c r="E5" s="7"/>
     </row>
     <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="A6" s="19"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="21"/>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="13"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
@@ -883,24 +887,26 @@
       <c r="C8" s="6">
         <v>10</v>
       </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="8">
+        <v>10</v>
+      </c>
       <c r="E8" s="7"/>
     </row>
     <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
+      <c r="A9" s="19"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="21"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
@@ -927,7 +933,9 @@
       <c r="C12" s="6">
         <v>1</v>
       </c>
-      <c r="D12" s="9"/>
+      <c r="D12" s="9">
+        <v>1</v>
+      </c>
       <c r="E12" s="10"/>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1032,20 +1040,20 @@
       <c r="E19" s="10"/>
     </row>
     <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="19"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="24"/>
     </row>
     <row r="21" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="13"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="18"/>
     </row>
     <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
@@ -1130,20 +1138,20 @@
       <c r="E27" s="10"/>
     </row>
     <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="19"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="24"/>
     </row>
     <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="13"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="18"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
@@ -1217,20 +1225,20 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="14"/>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="16"/>
+      <c r="A35" s="19"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="21"/>
     </row>
     <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="13"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="18"/>
     </row>
     <row r="37" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
@@ -1263,21 +1271,21 @@
       <c r="E38" s="10"/>
     </row>
     <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="17"/>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="19"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="24"/>
     </row>
     <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="13"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="18"/>
     </row>
     <row r="42" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
@@ -1289,7 +1297,9 @@
       <c r="C42" s="6">
         <v>2</v>
       </c>
-      <c r="D42" s="9"/>
+      <c r="D42" s="9">
+        <v>2</v>
+      </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1302,7 +1312,9 @@
       <c r="C43" s="6">
         <v>2</v>
       </c>
-      <c r="D43" s="9"/>
+      <c r="D43" s="9">
+        <v>2</v>
+      </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1315,7 +1327,9 @@
       <c r="C44" s="6">
         <v>2</v>
       </c>
-      <c r="D44" s="9"/>
+      <c r="D44" s="9">
+        <v>2</v>
+      </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1362,20 +1376,20 @@
       <c r="E47" s="7"/>
     </row>
     <row r="48" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="14"/>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="16"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="21"/>
     </row>
     <row r="49" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
+      <c r="A49" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="13"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="18"/>
     </row>
     <row r="50" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
@@ -1387,7 +1401,9 @@
       <c r="C50" s="6">
         <v>2</v>
       </c>
-      <c r="D50" s="9"/>
+      <c r="D50" s="9">
+        <v>2</v>
+      </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1400,7 +1416,9 @@
       <c r="C51" s="6">
         <v>1</v>
       </c>
-      <c r="D51" s="9"/>
+      <c r="D51" s="9">
+        <v>1</v>
+      </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1413,24 +1431,26 @@
       <c r="C52" s="6">
         <v>2</v>
       </c>
-      <c r="D52" s="9"/>
+      <c r="D52" s="9">
+        <v>2</v>
+      </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="17"/>
-      <c r="B53" s="18"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="18"/>
-      <c r="E53" s="19"/>
+      <c r="A53" s="22"/>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="24"/>
     </row>
     <row r="54" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="11" t="s">
+      <c r="A54" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="12"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="13"/>
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="18"/>
     </row>
     <row r="55" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
@@ -1442,7 +1462,9 @@
       <c r="C55" s="6">
         <v>2</v>
       </c>
-      <c r="D55" s="8"/>
+      <c r="D55" s="8">
+        <v>2</v>
+      </c>
       <c r="E55" s="7"/>
     </row>
     <row r="56" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1455,22 +1477,24 @@
       <c r="C56" s="6">
         <v>3</v>
       </c>
-      <c r="D56" s="8"/>
+      <c r="D56" s="8">
+        <v>3</v>
+      </c>
       <c r="E56" s="7"/>
     </row>
     <row r="57" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="14"/>
-      <c r="B57" s="15"/>
-      <c r="C57" s="15"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="16"/>
+      <c r="A57" s="19"/>
+      <c r="B57" s="20"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="21"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="20" t="s">
+      <c r="A58" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="21"/>
-      <c r="C58" s="21"/>
+      <c r="B58" s="12"/>
+      <c r="C58" s="12"/>
       <c r="D58" s="8"/>
       <c r="E58" s="7"/>
     </row>
@@ -1500,7 +1524,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" s="10"/>
     </row>
@@ -1568,7 +1592,9 @@
       <c r="C65" s="6">
         <v>1</v>
       </c>
-      <c r="D65" s="9"/>
+      <c r="D65" s="9">
+        <v>1</v>
+      </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1607,7 +1633,9 @@
       <c r="C68" s="6">
         <v>2</v>
       </c>
-      <c r="D68" s="9"/>
+      <c r="D68" s="9">
+        <v>2</v>
+      </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1624,18 +1652,18 @@
       <c r="E69" s="10"/>
     </row>
     <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="22"/>
-      <c r="B70" s="21"/>
-      <c r="C70" s="21"/>
+      <c r="A70" s="13"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="12"/>
       <c r="D70" s="8"/>
       <c r="E70" s="7"/>
     </row>
     <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="20" t="s">
+      <c r="A71" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="21"/>
-      <c r="C71" s="21"/>
+      <c r="B71" s="12"/>
+      <c r="C71" s="12"/>
       <c r="D71" s="8"/>
       <c r="E71" s="7"/>
     </row>
@@ -1677,7 +1705,7 @@
       <c r="E74" s="10"/>
     </row>
     <row r="75" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="23" t="s">
+      <c r="A75" s="14" t="s">
         <v>73</v>
       </c>
       <c r="B75" s="6"/>
@@ -1716,24 +1744,25 @@
       <c r="E79" s="10"/>
     </row>
     <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="20" t="s">
+      <c r="A80" s="11" t="s">
         <v>74</v>
       </c>
       <c r="B80" s="6"/>
-      <c r="C80" s="24"/>
+      <c r="C80" s="15"/>
       <c r="D80" s="9">
         <f>SUM(D1:D79)</f>
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="E80" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A28:E28"/>
@@ -1741,12 +1770,11 @@
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A54:E54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated readme link, project marking, and loaddata for edge case
</commit_message>
<xml_diff>
--- a/projectMarkingSoFar.xlsx
+++ b/projectMarkingSoFar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soljt\Documents\COSC 304\cosc304-project-group1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E6956F-9451-468D-95E7-9B2A10AF4869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A147DD8F-610E-4250-A417-01DB00E99BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{24B39AA9-47B0-4981-9C08-9EA32D2EDF33}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{24B39AA9-47B0-4981-9C08-9EA32D2EDF33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="56">
   <si>
     <t>Final Overall System Features</t>
   </si>
@@ -99,15 +99,9 @@
     <t>Page header shows current logged in user</t>
   </si>
   <si>
-    <t>Dynamic products on page based on sales</t>
-  </si>
-  <si>
     <t>Improved UI (user-friendly, images, etc.)</t>
   </si>
   <si>
-    <t>Product recommendation based on user</t>
-  </si>
-  <si>
     <t>Shopping Cart (up to 8 total points)</t>
   </si>
   <si>
@@ -117,39 +111,18 @@
     <t>View shopping cart</t>
   </si>
   <si>
-    <t>Update quantity (with data validation)</t>
-  </si>
-  <si>
-    <t>Remove item from shopping cart</t>
-  </si>
-  <si>
     <t>Improved formatting/UI (e.g. in header bar)</t>
   </si>
   <si>
-    <t>Cart stored in database between sessions</t>
-  </si>
-  <si>
     <t>Checkout (up to 9 total points)</t>
   </si>
   <si>
     <t>Checkout with customer id</t>
   </si>
   <si>
-    <t>Checkout with payment/shipment info</t>
-  </si>
-  <si>
     <t>Checkout with data validation</t>
   </si>
   <si>
-    <t>Multiple shipments per order supported</t>
-  </si>
-  <si>
-    <t>Note: Requires DB change.</t>
-  </si>
-  <si>
-    <t>Calculate taxes/shipping (by items/state)</t>
-  </si>
-  <si>
     <t>Product Detail Page (up to 2 total points)</t>
   </si>
   <si>
@@ -174,9 +147,6 @@
     <t>Login/logout</t>
   </si>
   <si>
-    <t>Register user/Forgot password email</t>
-  </si>
-  <si>
     <t>Page listing all orders for user</t>
   </si>
   <si>
@@ -216,9 +186,6 @@
     <t>List report showing total sales/orders</t>
   </si>
   <si>
-    <t>Report with a graph</t>
-  </si>
-  <si>
     <t>Add new product</t>
   </si>
   <si>
@@ -228,34 +195,10 @@
     <t>Change order status/ship order</t>
   </si>
   <si>
-    <t>Upload a photo to file system for product</t>
-  </si>
-  <si>
-    <t>OR: Upload a photo to database for product</t>
-  </si>
-  <si>
     <t>Database restore with SQL script</t>
   </si>
   <si>
     <t>Add/update warehouse, customer</t>
-  </si>
-  <si>
-    <t>Database System/General</t>
-  </si>
-  <si>
-    <t>Implement some validation using triggers</t>
-  </si>
-  <si>
-    <t>Use AJAX for some pages</t>
-  </si>
-  <si>
-    <t>User interface and navigation/usability</t>
-  </si>
-  <si>
-    <t>Up to 5</t>
-  </si>
-  <si>
-    <t>Others (your suggestions)</t>
   </si>
   <si>
     <t>Total: (out of 50 with maximum of 10 bonus marks. i.e. 60 points out of 50 is max.)</t>
@@ -265,7 +208,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,13 +235,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -396,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -436,9 +372,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -784,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0290CEB6-C15E-40D4-9522-224449852840}">
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="74.7109375" bestFit="1" customWidth="1"/>
@@ -808,13 +741,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="21"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="20"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -862,20 +795,20 @@
       <c r="E5" s="7"/>
     </row>
     <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="24"/>
+      <c r="A6" s="21"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="20"/>
     </row>
     <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
@@ -893,20 +826,20 @@
       <c r="E8" s="7"/>
     </row>
     <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="24"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="21"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="20"/>
     </row>
     <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
@@ -994,7 +927,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="10"/>
     </row>
@@ -1008,59 +941,63 @@
       <c r="C17" s="6">
         <v>2</v>
       </c>
-      <c r="D17" s="9"/>
+      <c r="D17" s="9">
+        <v>2</v>
+      </c>
       <c r="E17" s="10"/>
     </row>
     <row r="18" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="15"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17"/>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="6">
-        <v>2</v>
-      </c>
-      <c r="D18" s="9">
-        <v>2</v>
-      </c>
-      <c r="E18" s="10"/>
-    </row>
-    <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20"/>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="6">
-        <v>4</v>
-      </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="18"/>
+      <c r="B20" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9">
+        <v>1</v>
+      </c>
+      <c r="E20" s="10"/>
     </row>
     <row r="21" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="21"/>
+      <c r="B21" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="9">
+        <v>1</v>
+      </c>
+      <c r="E21" s="10"/>
     </row>
     <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C22" s="6">
         <v>1</v>
@@ -1071,178 +1008,162 @@
       <c r="E22" s="10"/>
     </row>
     <row r="23" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="15"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="17"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="6">
-        <v>1</v>
-      </c>
-      <c r="D23" s="9">
-        <v>1</v>
-      </c>
-      <c r="E23" s="10"/>
-    </row>
-    <row r="24" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="6">
-        <v>1</v>
-      </c>
-      <c r="D24" s="9"/>
-      <c r="E24" s="10"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="20"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C25" s="6">
         <v>1</v>
       </c>
-      <c r="D25" s="9"/>
+      <c r="D25" s="9">
+        <v>1</v>
+      </c>
       <c r="E25" s="10"/>
     </row>
     <row r="26" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C26" s="6">
-        <v>1</v>
-      </c>
-      <c r="D26" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="D26" s="9">
+        <v>2</v>
+      </c>
       <c r="E26" s="10"/>
     </row>
     <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="21"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="20"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="6">
-        <v>3</v>
-      </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
-    </row>
-    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="18"/>
-    </row>
-    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="21"/>
+      <c r="B29" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="6">
+        <v>1</v>
+      </c>
+      <c r="D29" s="9">
+        <v>1</v>
+      </c>
+      <c r="E29" s="10"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1</v>
+      </c>
+      <c r="D30" s="9">
+        <v>1</v>
+      </c>
+      <c r="E30" s="10"/>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="15"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="17"/>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C30" s="6">
-        <v>1</v>
-      </c>
-      <c r="D30" s="9">
-        <v>1</v>
-      </c>
-      <c r="E30" s="10"/>
-    </row>
-    <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="20"/>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B34" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="6">
-        <v>2</v>
-      </c>
-      <c r="D31" s="9"/>
-      <c r="E31" s="10"/>
-    </row>
-    <row r="32" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
+      <c r="C34" s="6">
+        <v>2</v>
+      </c>
+      <c r="D34" s="9">
+        <v>2</v>
+      </c>
+      <c r="E34" s="10"/>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="6">
-        <v>2</v>
-      </c>
-      <c r="D32" s="9"/>
-      <c r="E32" s="10"/>
-    </row>
-    <row r="33" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="C35" s="6">
+        <v>2</v>
+      </c>
+      <c r="D35" s="9">
+        <v>2</v>
+      </c>
+      <c r="E35" s="10"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="6">
-        <v>2</v>
-      </c>
-      <c r="D33" s="9"/>
-      <c r="E33" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" s="6">
-        <v>2</v>
-      </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="22"/>
-      <c r="B35" s="23"/>
-      <c r="C35" s="23"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="24"/>
-    </row>
-    <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="21"/>
+      <c r="B36" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="6">
+        <v>2</v>
+      </c>
+      <c r="D36" s="9">
+        <v>2</v>
+      </c>
+      <c r="E36" s="10"/>
     </row>
     <row r="37" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>7</v>
@@ -1257,7 +1178,7 @@
     </row>
     <row r="38" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>7</v>
@@ -1265,49 +1186,63 @@
       <c r="C38" s="6">
         <v>1</v>
       </c>
-      <c r="D38" s="9">
-        <v>1</v>
-      </c>
-      <c r="E38" s="10"/>
+      <c r="D38" s="8">
+        <v>1</v>
+      </c>
+      <c r="E38" s="7"/>
     </row>
     <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="16"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="18"/>
-    </row>
-    <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+      <c r="A39" s="21"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="23"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="20"/>
+    </row>
     <row r="41" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="21"/>
+      <c r="A41" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="6">
+        <v>2</v>
+      </c>
+      <c r="D41" s="9">
+        <v>2</v>
+      </c>
+      <c r="E41" s="10"/>
     </row>
     <row r="42" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C42" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D42" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C43" s="6">
         <v>2</v>
@@ -1318,100 +1253,88 @@
       <c r="E43" s="10"/>
     </row>
     <row r="44" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C44" s="6">
-        <v>2</v>
-      </c>
-      <c r="D44" s="9">
-        <v>2</v>
-      </c>
-      <c r="E44" s="10"/>
+      <c r="A44" s="15"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="17"/>
     </row>
     <row r="45" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C45" s="6">
-        <v>1</v>
-      </c>
-      <c r="D45" s="9">
-        <v>1</v>
-      </c>
-      <c r="E45" s="10"/>
+      <c r="A45" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" s="19"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="20"/>
     </row>
     <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="C46" s="6">
-        <v>4</v>
-      </c>
-      <c r="D46" s="9"/>
-      <c r="E46" s="10"/>
+        <v>2</v>
+      </c>
+      <c r="D46" s="8">
+        <v>2</v>
+      </c>
+      <c r="E46" s="7"/>
     </row>
     <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C47" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D47" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E47" s="7"/>
     </row>
     <row r="48" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="22"/>
-      <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
-      <c r="D48" s="23"/>
-      <c r="E48" s="24"/>
+      <c r="A48" s="21"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="23"/>
     </row>
     <row r="49" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="21"/>
+      <c r="A49" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="7"/>
     </row>
     <row r="50" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C50" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C51" s="6">
         <v>1</v>
@@ -1423,359 +1346,128 @@
     </row>
     <row r="52" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="6">
+        <v>1</v>
+      </c>
+      <c r="D52" s="9">
+        <v>1</v>
+      </c>
+      <c r="E52" s="10"/>
+    </row>
+    <row r="53" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C53" s="6">
+        <v>2</v>
+      </c>
+      <c r="D53" s="9">
+        <v>2</v>
+      </c>
+      <c r="E53" s="10"/>
+    </row>
+    <row r="54" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C52" s="6">
-        <v>2</v>
-      </c>
-      <c r="D52" s="9">
-        <v>2</v>
-      </c>
-      <c r="E52" s="10"/>
-    </row>
-    <row r="53" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="16"/>
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="18"/>
-    </row>
-    <row r="54" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="21"/>
+      <c r="B54" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C54" s="6">
+        <v>2</v>
+      </c>
+      <c r="D54" s="9">
+        <v>2</v>
+      </c>
+      <c r="E54" s="10"/>
     </row>
     <row r="55" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="C55" s="6">
-        <v>2</v>
-      </c>
-      <c r="D55" s="8">
-        <v>2</v>
-      </c>
-      <c r="E55" s="7"/>
+        <v>1</v>
+      </c>
+      <c r="D55" s="9">
+        <v>1</v>
+      </c>
+      <c r="E55" s="10"/>
     </row>
     <row r="56" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C56" s="6">
-        <v>3</v>
-      </c>
-      <c r="D56" s="8">
-        <v>3</v>
-      </c>
-      <c r="E56" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D56" s="9">
+        <v>2</v>
+      </c>
+      <c r="E56" s="10"/>
     </row>
     <row r="57" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="22"/>
-      <c r="B57" s="23"/>
-      <c r="C57" s="23"/>
-      <c r="D57" s="23"/>
-      <c r="E57" s="24"/>
+      <c r="A57" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C57" s="6">
+        <v>2</v>
+      </c>
+      <c r="D57" s="9">
+        <v>2</v>
+      </c>
+      <c r="E57" s="10"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="11" t="s">
-        <v>56</v>
-      </c>
+      <c r="A58" s="13"/>
       <c r="B58" s="12"/>
       <c r="C58" s="12"/>
       <c r="D58" s="8"/>
       <c r="E58" s="7"/>
     </row>
     <row r="59" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C59" s="6">
-        <v>1</v>
-      </c>
+      <c r="A59" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B59" s="6"/>
+      <c r="C59" s="14"/>
       <c r="D59" s="9">
-        <v>1</v>
+        <f>SUM(D1:D58)</f>
+        <v>66</v>
       </c>
       <c r="E59" s="10"/>
-    </row>
-    <row r="60" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C60" s="6">
-        <v>1</v>
-      </c>
-      <c r="D60" s="9">
-        <v>1</v>
-      </c>
-      <c r="E60" s="10"/>
-    </row>
-    <row r="61" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C61" s="6">
-        <v>1</v>
-      </c>
-      <c r="D61" s="9">
-        <v>1</v>
-      </c>
-      <c r="E61" s="10"/>
-    </row>
-    <row r="62" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C62" s="6">
-        <v>3</v>
-      </c>
-      <c r="D62" s="9"/>
-      <c r="E62" s="10"/>
-    </row>
-    <row r="63" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C63" s="6">
-        <v>2</v>
-      </c>
-      <c r="D63" s="9">
-        <v>2</v>
-      </c>
-      <c r="E63" s="10"/>
-    </row>
-    <row r="64" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C64" s="6">
-        <v>2</v>
-      </c>
-      <c r="D64" s="9">
-        <v>2</v>
-      </c>
-      <c r="E64" s="10"/>
-    </row>
-    <row r="65" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C65" s="6">
-        <v>1</v>
-      </c>
-      <c r="D65" s="9">
-        <v>1</v>
-      </c>
-      <c r="E65" s="10"/>
-    </row>
-    <row r="66" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C66" s="6">
-        <v>2</v>
-      </c>
-      <c r="D66" s="9"/>
-      <c r="E66" s="10"/>
-    </row>
-    <row r="67" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B67" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C67" s="6">
-        <v>4</v>
-      </c>
-      <c r="D67" s="9"/>
-      <c r="E67" s="10"/>
-    </row>
-    <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C68" s="6">
-        <v>2</v>
-      </c>
-      <c r="D68" s="9">
-        <v>2</v>
-      </c>
-      <c r="E68" s="10"/>
-    </row>
-    <row r="69" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B69" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C69" s="6">
-        <v>2</v>
-      </c>
-      <c r="D69" s="9">
-        <v>2</v>
-      </c>
-      <c r="E69" s="10"/>
-    </row>
-    <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="13"/>
-      <c r="B70" s="12"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="8"/>
-      <c r="E70" s="7"/>
-    </row>
-    <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B71" s="12"/>
-      <c r="C71" s="12"/>
-      <c r="D71" s="8"/>
-      <c r="E71" s="7"/>
-    </row>
-    <row r="72" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C72" s="6">
-        <v>2</v>
-      </c>
-      <c r="D72" s="9"/>
-      <c r="E72" s="10"/>
-    </row>
-    <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B73" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C73" s="6">
-        <v>4</v>
-      </c>
-      <c r="D73" s="9"/>
-      <c r="E73" s="10"/>
-    </row>
-    <row r="74" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B74" s="6"/>
-      <c r="C74" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D74" s="9"/>
-      <c r="E74" s="10"/>
-    </row>
-    <row r="75" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B75" s="6"/>
-      <c r="C75" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D75" s="9"/>
-      <c r="E75" s="10"/>
-    </row>
-    <row r="76" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="5"/>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6"/>
-      <c r="D76" s="9"/>
-      <c r="E76" s="10"/>
-    </row>
-    <row r="77" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="5"/>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="10"/>
-    </row>
-    <row r="78" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="5"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="6"/>
-      <c r="D78" s="9"/>
-      <c r="E78" s="10"/>
-    </row>
-    <row r="79" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="5"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="6"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="10"/>
-    </row>
-    <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="B80" s="6"/>
-      <c r="C80" s="15"/>
-      <c r="D80" s="9">
-        <f>SUM(D1:D79)</f>
-        <v>62</v>
-      </c>
-      <c r="E80" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A27:E27"/>
     <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A7:E7"/>

</xml_diff>